<commit_message>
Updated SAU_grids_kan25 model - 2026-07-24 19:14
</commit_message>
<xml_diff>
--- a/VerveStacks_SAU_grids_kan25/Sets-vervestacks.xlsx
+++ b/VerveStacks_SAU_grids_kan25/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_SAU_grids_kan25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98B17612-DF24-418D-942B-831B91339FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6269FF2E-15C3-407D-BD5A-6F2558473E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -367,7 +367,7 @@
     <t>p_w115168488-380_SAU</t>
   </si>
   <si>
-    <t>e_w115168488-380_SAU*</t>
+    <t>*[_]w115168488-380_SAU</t>
   </si>
   <si>
     <t>OR</t>
@@ -376,109 +376,109 @@
     <t>p_w900157271-380_SAU</t>
   </si>
   <si>
-    <t>e_w900157271-380_SAU*</t>
+    <t>*[_]w900157271-380_SAU</t>
   </si>
   <si>
     <t>p_w181132741-380_SAU</t>
   </si>
   <si>
-    <t>e_w181132741-380_SAU*</t>
+    <t>*[_]w181132741-380_SAU</t>
   </si>
   <si>
     <t>p_w198144511-230_SAU</t>
   </si>
   <si>
-    <t>e_w198144511-230_SAU*</t>
+    <t>*[_]w198144511-230_SAU</t>
   </si>
   <si>
     <t>p_w203627872-380_SAU</t>
   </si>
   <si>
-    <t>e_w203627872-380_SAU*</t>
+    <t>*[_]w203627872-380_SAU</t>
   </si>
   <si>
     <t>p_w204824991-380_SAU</t>
   </si>
   <si>
-    <t>e_w204824991-380_SAU*</t>
+    <t>*[_]w204824991-380_SAU</t>
   </si>
   <si>
     <t>p_w207785816-380_SAU</t>
   </si>
   <si>
-    <t>e_w207785816-380_SAU*</t>
+    <t>*[_]w207785816-380_SAU</t>
   </si>
   <si>
     <t>p_w1317464635-380_SAU</t>
   </si>
   <si>
-    <t>e_w1317464635-380_SAU*</t>
+    <t>*[_]w1317464635-380_SAU</t>
   </si>
   <si>
     <t>p_w524688755-380_SAU</t>
   </si>
   <si>
-    <t>e_w524688755-380_SAU*</t>
+    <t>*[_]w524688755-380_SAU</t>
   </si>
   <si>
     <t>p_w524938770-380_SAU</t>
   </si>
   <si>
-    <t>e_w524938770-380_SAU*</t>
+    <t>*[_]w524938770-380_SAU</t>
   </si>
   <si>
     <t>p_w582073817-380_SAU</t>
   </si>
   <si>
-    <t>e_w582073817-380_SAU*</t>
+    <t>*[_]w582073817-380_SAU</t>
   </si>
   <si>
     <t>p_w586137460-380_SAU</t>
   </si>
   <si>
-    <t>e_w586137460-380_SAU*</t>
+    <t>*[_]w586137460-380_SAU</t>
   </si>
   <si>
     <t>p_w597093579-380_SAU</t>
   </si>
   <si>
-    <t>e_w597093579-380_SAU*</t>
+    <t>*[_]w597093579-380_SAU</t>
   </si>
   <si>
     <t>p_w818080067-380_SAU</t>
   </si>
   <si>
-    <t>e_w818080067-380_SAU*</t>
+    <t>*[_]w818080067-380_SAU</t>
   </si>
   <si>
     <t>p_w818155745-380_SAU</t>
   </si>
   <si>
-    <t>e_w818155745-380_SAU*</t>
+    <t>*[_]w818155745-380_SAU</t>
   </si>
   <si>
     <t>p_w820233467-380_SAU</t>
   </si>
   <si>
-    <t>e_w820233467-380_SAU*</t>
+    <t>*[_]w820233467-380_SAU</t>
   </si>
   <si>
     <t>p_w899264357-380_SAU</t>
   </si>
   <si>
-    <t>e_w899264357-380_SAU*</t>
+    <t>*[_]w899264357-380_SAU</t>
   </si>
   <si>
     <t>p_SA12-380_SAU</t>
   </si>
   <si>
-    <t>e_SA12-380_SAU*</t>
+    <t>*[_]SA12-380_SAU</t>
   </si>
   <si>
     <t>p_SA4-380_SAU</t>
   </si>
   <si>
-    <t>e_SA4-380_SAU*</t>
+    <t>*[_]SA4-380_SAU</t>
   </si>
   <si>
     <t>rez_spv_SAU_001</t>
@@ -2109,7 +2109,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D10DC1F1-4C57-47A0-A46A-1A5C17C440CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BC79E2F-EAB4-4191-AB8A-E531B979C275}">
   <dimension ref="B9:E160"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>